<commit_message>
Update fee records and student codes
This commit adds two new student code registrations and updates term fee payment data for multiple students. It reflects new payments, balances, and fully paid entries in the 2026-2027 fee dataset.
</commit_message>
<xml_diff>
--- a/parent_codes.xlsx
+++ b/parent_codes.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="268">
   <si>
     <t>Code</t>
   </si>
@@ -94,6 +94,9 @@
     <t>ADEIRE1013</t>
   </si>
   <si>
+    <t>ADEMAR1126</t>
+  </si>
+  <si>
     <t>ADEMOD1027</t>
   </si>
   <si>
@@ -115,6 +118,9 @@
     <t>ADIAHN1029</t>
   </si>
   <si>
+    <t>AGUCHR1127</t>
+  </si>
+  <si>
     <t>AKAMIC1031</t>
   </si>
   <si>
@@ -463,6 +469,9 @@
     <t>ADEDAMOLA IREMIDE</t>
   </si>
   <si>
+    <t>ADEDINI MARY OLUWATOFUNMI</t>
+  </si>
+  <si>
     <t>ADEYEMI MODADEOBA GBOLAHAN</t>
   </si>
   <si>
@@ -484,6 +493,9 @@
     <t>ADIGUN AHNAF ARAOLA</t>
   </si>
   <si>
+    <t>AGUNBIADE CHRISTIANAH OLUWAKEMI</t>
+  </si>
+  <si>
     <t>AKANDE MICHELLE OREOFE</t>
   </si>
   <si>
@@ -794,6 +806,9 @@
   </si>
   <si>
     <t>PRIMARY 5</t>
+  </si>
+  <si>
+    <t>JUNIOR SECONDARY SCHOOL 1</t>
   </si>
   <si>
     <t>CRECHE</t>
@@ -1134,7 +1149,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1153,10 +1168,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C2" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1164,10 +1179,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C3" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1175,10 +1190,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C4" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1186,10 +1201,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C5" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1197,10 +1212,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C6" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1208,10 +1223,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C7" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1219,10 +1234,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C8" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1230,10 +1245,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C9" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1241,10 +1256,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C10" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1252,10 +1267,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C11" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1263,10 +1278,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C12" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1274,10 +1289,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C13" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1285,10 +1300,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C14" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1296,10 +1311,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C15" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1307,10 +1322,10 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C16" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1318,10 +1333,10 @@
         <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C17" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1329,10 +1344,10 @@
         <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C18" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1340,10 +1355,10 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C19" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1351,10 +1366,10 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C20" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1362,10 +1377,10 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C21" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1373,10 +1388,10 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C22" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1384,10 +1399,10 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C23" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1395,10 +1410,10 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C24" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1406,10 +1421,10 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C25" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1417,10 +1432,10 @@
         <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C26" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1428,10 +1443,10 @@
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C27" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1439,10 +1454,10 @@
         <v>29</v>
       </c>
       <c r="B28" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C28" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1450,10 +1465,10 @@
         <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C29" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1461,10 +1476,10 @@
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C30" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1472,10 +1487,10 @@
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C31" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1483,7 +1498,7 @@
         <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C32" t="s">
         <v>260</v>
@@ -1494,10 +1509,10 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C33" t="s">
-        <v>248</v>
+        <v>264</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1505,10 +1520,10 @@
         <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C34" t="s">
-        <v>249</v>
+        <v>265</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1516,10 +1531,10 @@
         <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C35" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -1527,10 +1542,10 @@
         <v>37</v>
       </c>
       <c r="B36" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C36" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1538,10 +1553,10 @@
         <v>38</v>
       </c>
       <c r="B37" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C37" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1549,10 +1564,10 @@
         <v>39</v>
       </c>
       <c r="B38" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C38" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -1560,10 +1575,10 @@
         <v>40</v>
       </c>
       <c r="B39" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C39" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -1571,10 +1586,10 @@
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C40" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1582,10 +1597,10 @@
         <v>42</v>
       </c>
       <c r="B41" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C41" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1593,10 +1608,10 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C42" t="s">
-        <v>250</v>
+        <v>261</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1604,10 +1619,10 @@
         <v>44</v>
       </c>
       <c r="B43" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C43" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -1615,10 +1630,10 @@
         <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C44" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -1626,10 +1641,10 @@
         <v>46</v>
       </c>
       <c r="B45" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C45" t="s">
-        <v>250</v>
+        <v>261</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -1637,10 +1652,10 @@
         <v>47</v>
       </c>
       <c r="B46" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C46" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -1648,10 +1663,10 @@
         <v>48</v>
       </c>
       <c r="B47" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C47" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -1659,10 +1674,10 @@
         <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C48" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -1670,10 +1685,10 @@
         <v>50</v>
       </c>
       <c r="B49" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C49" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1681,10 +1696,10 @@
         <v>51</v>
       </c>
       <c r="B50" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C50" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -1692,10 +1707,10 @@
         <v>52</v>
       </c>
       <c r="B51" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C51" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -1703,10 +1718,10 @@
         <v>53</v>
       </c>
       <c r="B52" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C52" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -1714,10 +1729,10 @@
         <v>54</v>
       </c>
       <c r="B53" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C53" t="s">
-        <v>252</v>
+        <v>263</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -1725,10 +1740,10 @@
         <v>55</v>
       </c>
       <c r="B54" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C54" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1736,10 +1751,10 @@
         <v>56</v>
       </c>
       <c r="B55" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C55" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -1747,10 +1762,10 @@
         <v>57</v>
       </c>
       <c r="B56" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C56" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1758,10 +1773,10 @@
         <v>58</v>
       </c>
       <c r="B57" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C57" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1769,10 +1784,10 @@
         <v>59</v>
       </c>
       <c r="B58" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C58" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -1780,10 +1795,10 @@
         <v>60</v>
       </c>
       <c r="B59" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C59" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1791,10 +1806,10 @@
         <v>61</v>
       </c>
       <c r="B60" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C60" t="s">
-        <v>248</v>
+        <v>262</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1802,10 +1817,10 @@
         <v>62</v>
       </c>
       <c r="B61" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C61" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -1813,10 +1828,10 @@
         <v>63</v>
       </c>
       <c r="B62" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C62" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -1824,10 +1839,10 @@
         <v>64</v>
       </c>
       <c r="B63" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C63" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -1835,10 +1850,10 @@
         <v>65</v>
       </c>
       <c r="B64" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C64" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1846,10 +1861,10 @@
         <v>66</v>
       </c>
       <c r="B65" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C65" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -1857,10 +1872,10 @@
         <v>67</v>
       </c>
       <c r="B66" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C66" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -1868,10 +1883,10 @@
         <v>68</v>
       </c>
       <c r="B67" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C67" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -1879,10 +1894,10 @@
         <v>69</v>
       </c>
       <c r="B68" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C68" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -1890,10 +1905,10 @@
         <v>70</v>
       </c>
       <c r="B69" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C69" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -1901,10 +1916,10 @@
         <v>71</v>
       </c>
       <c r="B70" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C70" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -1912,10 +1927,10 @@
         <v>72</v>
       </c>
       <c r="B71" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C71" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -1923,10 +1938,10 @@
         <v>73</v>
       </c>
       <c r="B72" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C72" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -1934,10 +1949,10 @@
         <v>74</v>
       </c>
       <c r="B73" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C73" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -1945,10 +1960,10 @@
         <v>75</v>
       </c>
       <c r="B74" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C74" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -1956,10 +1971,10 @@
         <v>76</v>
       </c>
       <c r="B75" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C75" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -1967,10 +1982,10 @@
         <v>77</v>
       </c>
       <c r="B76" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C76" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="77" spans="1:3">
@@ -1978,10 +1993,10 @@
         <v>78</v>
       </c>
       <c r="B77" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C77" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
     </row>
     <row r="78" spans="1:3">
@@ -1989,10 +2004,10 @@
         <v>79</v>
       </c>
       <c r="B78" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C78" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="79" spans="1:3">
@@ -2000,10 +2015,10 @@
         <v>80</v>
       </c>
       <c r="B79" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C79" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -2011,10 +2026,10 @@
         <v>81</v>
       </c>
       <c r="B80" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C80" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -2022,10 +2037,10 @@
         <v>82</v>
       </c>
       <c r="B81" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C81" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -2033,10 +2048,10 @@
         <v>83</v>
       </c>
       <c r="B82" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C82" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -2044,10 +2059,10 @@
         <v>84</v>
       </c>
       <c r="B83" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C83" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -2055,10 +2070,10 @@
         <v>85</v>
       </c>
       <c r="B84" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C84" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -2066,7 +2081,10 @@
         <v>86</v>
       </c>
       <c r="B85" t="s">
-        <v>208</v>
+        <v>210</v>
+      </c>
+      <c r="C85" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -2074,10 +2092,10 @@
         <v>87</v>
       </c>
       <c r="B86" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C86" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -2085,10 +2103,7 @@
         <v>88</v>
       </c>
       <c r="B87" t="s">
-        <v>210</v>
-      </c>
-      <c r="C87" t="s">
-        <v>256</v>
+        <v>212</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -2096,10 +2111,10 @@
         <v>89</v>
       </c>
       <c r="B88" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C88" t="s">
-        <v>248</v>
+        <v>267</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -2107,10 +2122,10 @@
         <v>90</v>
       </c>
       <c r="B89" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C89" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -2118,10 +2133,10 @@
         <v>91</v>
       </c>
       <c r="B90" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C90" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -2129,10 +2144,10 @@
         <v>92</v>
       </c>
       <c r="B91" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C91" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="92" spans="1:3">
@@ -2140,10 +2155,10 @@
         <v>93</v>
       </c>
       <c r="B92" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C92" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -2151,10 +2166,10 @@
         <v>94</v>
       </c>
       <c r="B93" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C93" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -2162,10 +2177,10 @@
         <v>95</v>
       </c>
       <c r="B94" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C94" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -2173,10 +2188,10 @@
         <v>96</v>
       </c>
       <c r="B95" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C95" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -2184,10 +2199,10 @@
         <v>97</v>
       </c>
       <c r="B96" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C96" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -2195,10 +2210,10 @@
         <v>98</v>
       </c>
       <c r="B97" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C97" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -2206,10 +2221,10 @@
         <v>99</v>
       </c>
       <c r="B98" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C98" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
     </row>
     <row r="99" spans="1:3">
@@ -2217,10 +2232,10 @@
         <v>100</v>
       </c>
       <c r="B99" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C99" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -2228,10 +2243,10 @@
         <v>101</v>
       </c>
       <c r="B100" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C100" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="101" spans="1:3">
@@ -2239,10 +2254,10 @@
         <v>102</v>
       </c>
       <c r="B101" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C101" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -2250,10 +2265,10 @@
         <v>103</v>
       </c>
       <c r="B102" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C102" t="s">
-        <v>249</v>
+        <v>266</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -2261,10 +2276,10 @@
         <v>104</v>
       </c>
       <c r="B103" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C103" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="104" spans="1:3">
@@ -2272,7 +2287,7 @@
         <v>105</v>
       </c>
       <c r="B104" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C104" t="s">
         <v>253</v>
@@ -2283,10 +2298,10 @@
         <v>106</v>
       </c>
       <c r="B105" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C105" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
     </row>
     <row r="106" spans="1:3">
@@ -2294,10 +2309,10 @@
         <v>107</v>
       </c>
       <c r="B106" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C106" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -2305,10 +2320,10 @@
         <v>108</v>
       </c>
       <c r="B107" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C107" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -2316,10 +2331,10 @@
         <v>109</v>
       </c>
       <c r="B108" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C108" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -2327,10 +2342,10 @@
         <v>110</v>
       </c>
       <c r="B109" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C109" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -2338,10 +2353,10 @@
         <v>111</v>
       </c>
       <c r="B110" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C110" t="s">
-        <v>251</v>
+        <v>265</v>
       </c>
     </row>
     <row r="111" spans="1:3">
@@ -2349,10 +2364,10 @@
         <v>112</v>
       </c>
       <c r="B111" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C111" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -2360,10 +2375,10 @@
         <v>113</v>
       </c>
       <c r="B112" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C112" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -2371,10 +2386,10 @@
         <v>114</v>
       </c>
       <c r="B113" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C113" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -2382,10 +2397,10 @@
         <v>115</v>
       </c>
       <c r="B114" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C114" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -2393,10 +2408,10 @@
         <v>116</v>
       </c>
       <c r="B115" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C115" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -2404,10 +2419,10 @@
         <v>117</v>
       </c>
       <c r="B116" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C116" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="117" spans="1:3">
@@ -2415,10 +2430,10 @@
         <v>118</v>
       </c>
       <c r="B117" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C117" t="s">
-        <v>252</v>
+        <v>266</v>
       </c>
     </row>
     <row r="118" spans="1:3">
@@ -2426,10 +2441,10 @@
         <v>119</v>
       </c>
       <c r="B118" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C118" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -2437,10 +2452,10 @@
         <v>120</v>
       </c>
       <c r="B119" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C119" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
     </row>
     <row r="120" spans="1:3">
@@ -2448,10 +2463,10 @@
         <v>121</v>
       </c>
       <c r="B120" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C120" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="121" spans="1:3">
@@ -2459,10 +2474,10 @@
         <v>122</v>
       </c>
       <c r="B121" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C121" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
     </row>
     <row r="122" spans="1:3">
@@ -2470,10 +2485,10 @@
         <v>123</v>
       </c>
       <c r="B122" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C122" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
     </row>
     <row r="123" spans="1:3">
@@ -2481,10 +2496,10 @@
         <v>124</v>
       </c>
       <c r="B123" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C123" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="124" spans="1:3">
@@ -2492,10 +2507,32 @@
         <v>125</v>
       </c>
       <c r="B124" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C124" t="s">
-        <v>248</v>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3">
+      <c r="A125" t="s">
+        <v>126</v>
+      </c>
+      <c r="B125" t="s">
+        <v>250</v>
+      </c>
+      <c r="C125" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3">
+      <c r="A126" t="s">
+        <v>127</v>
+      </c>
+      <c r="B126" t="s">
+        <v>251</v>
+      </c>
+      <c r="C126" t="s">
+        <v>252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update fee data and add new student codes
Add multiple new code mappings to code_registry.json and add/update corresponding records in students_1st_term.json. Normalize numeric/detail fields (e.g. "0.0" -> "0"), add entries for ADEMAR1128, EMIOBA1129, EMIMAR1130, FASABD1131, FASABD1132, ISMMAB1133, MORPRI1134, OGOJOS1135, OYIIBU1136, ISAEYI1137, and correct totals, payments, balances and class assignments for several students. Also update parent_codes.xlsx and 2026 - 2027 FEE.xlsx binary files.
</commit_message>
<xml_diff>
--- a/parent_codes.xlsx
+++ b/parent_codes.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="285">
   <si>
     <t>Code</t>
   </si>
@@ -97,6 +97,9 @@
     <t>ADEMAR1126</t>
   </si>
   <si>
+    <t>ADEMAR1128</t>
+  </si>
+  <si>
     <t>ADEMOD1027</t>
   </si>
   <si>
@@ -175,6 +178,12 @@
     <t>EDEZEN1048</t>
   </si>
   <si>
+    <t>EMIMAR1130</t>
+  </si>
+  <si>
+    <t>EMIOBA1129</t>
+  </si>
+  <si>
     <t>EMMRUT1049</t>
   </si>
   <si>
@@ -190,10 +199,10 @@
     <t>FAGASE1053</t>
   </si>
   <si>
-    <t>FAS1122</t>
-  </si>
-  <si>
-    <t>FAS1123</t>
+    <t>FASABD1131</t>
+  </si>
+  <si>
+    <t>FASABD1132</t>
   </si>
   <si>
     <t>FEYJAD1054</t>
@@ -220,6 +229,12 @@
     <t>IGEOLU1061</t>
   </si>
   <si>
+    <t>ISAEYI1137</t>
+  </si>
+  <si>
+    <t>ISMMAB1133</t>
+  </si>
+  <si>
     <t>ISSIMO1062</t>
   </si>
   <si>
@@ -256,6 +271,9 @@
     <t>KONUMA1072</t>
   </si>
   <si>
+    <t>MORPRI1134</t>
+  </si>
+  <si>
     <t>MOSHEP1074</t>
   </si>
   <si>
@@ -277,6 +295,9 @@
     <t>OBETAI1079</t>
   </si>
   <si>
+    <t>OGOJOS1135</t>
+  </si>
+  <si>
     <t>OGUOLU1124</t>
   </si>
   <si>
@@ -355,6 +376,9 @@
     <t>OYEISA1104</t>
   </si>
   <si>
+    <t>OYIIBU1136</t>
+  </si>
+  <si>
     <t>PETFAV1106</t>
   </si>
   <si>
@@ -472,6 +496,9 @@
     <t>ADEDINI MARY OLUWATOFUNMI</t>
   </si>
   <si>
+    <t>ADEBOWALE MARTIN</t>
+  </si>
+  <si>
     <t>ADEYEMI MODADEOBA GBOLAHAN</t>
   </si>
   <si>
@@ -550,6 +577,12 @@
     <t>EDEM ZENITH AYOKUNNUMI</t>
   </si>
   <si>
+    <t>EMIOLA MARVELLOUS QUADRI</t>
+  </si>
+  <si>
+    <t>EMIOLA OBALOLUWA MUHAMMED</t>
+  </si>
+  <si>
     <t>EMMANUEL RUTH OLADIPUPO</t>
   </si>
   <si>
@@ -565,7 +598,10 @@
     <t>FAGBAYI ASEOLUWA JOSHUA</t>
   </si>
   <si>
-    <t>FASASI</t>
+    <t>FASASI ABDULSAMAD</t>
+  </si>
+  <si>
+    <t>FASASI ABDULLATEEF</t>
   </si>
   <si>
     <t>FEYIJIMI JADEN OLAOLUWA</t>
@@ -592,6 +628,12 @@
     <t>IGE OLUWAFEMI BRIGHT</t>
   </si>
   <si>
+    <t>ISAAC EYINJUOLUWA HERITAGE</t>
+  </si>
+  <si>
+    <t>ISMAIL MABUB</t>
+  </si>
+  <si>
     <t>ISSAH IMOLE</t>
   </si>
   <si>
@@ -628,6 +670,9 @@
     <t>KONNEH UMAR IREBAMI</t>
   </si>
   <si>
+    <t>MORADEYO PRISCILLA OLUWADARASIMI</t>
+  </si>
+  <si>
     <t>MOSES HEPHZIBAH TOLUWALASE</t>
   </si>
   <si>
@@ -649,6 +694,9 @@
     <t>OBEY TAIWO EYITAYO</t>
   </si>
   <si>
+    <t>OGOOLUWADE JOSEPH</t>
+  </si>
+  <si>
     <t>OGUNSANYA OLUWAFERANMI BLESSED</t>
   </si>
   <si>
@@ -725,6 +773,9 @@
   </si>
   <si>
     <t>OYETUNJI ISAAC ORINAYO</t>
+  </si>
+  <si>
+    <t>OYINLOLA IBUKUNOLUWA VICTOR</t>
   </si>
   <si>
     <t>PETER FAVOUR ELIANA</t>
@@ -1149,7 +1200,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1168,10 +1219,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="C2" t="s">
-        <v>252</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1179,10 +1230,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="C3" t="s">
-        <v>253</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1190,10 +1241,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="C4" t="s">
-        <v>254</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1201,10 +1252,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="C5" t="s">
-        <v>255</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1212,10 +1263,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="C6" t="s">
-        <v>252</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1223,10 +1274,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="C7" t="s">
-        <v>256</v>
+        <v>273</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1234,10 +1285,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C8" t="s">
-        <v>257</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1245,10 +1296,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="C9" t="s">
-        <v>256</v>
+        <v>273</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1256,10 +1307,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C10" t="s">
-        <v>256</v>
+        <v>273</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1267,10 +1318,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="C11" t="s">
-        <v>256</v>
+        <v>273</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1278,10 +1329,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C12" t="s">
-        <v>255</v>
+        <v>272</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1289,10 +1340,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="C13" t="s">
-        <v>257</v>
+        <v>274</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1300,10 +1351,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="C14" t="s">
-        <v>254</v>
+        <v>271</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1311,10 +1362,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="C15" t="s">
-        <v>253</v>
+        <v>270</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1322,10 +1373,10 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="C16" t="s">
-        <v>257</v>
+        <v>274</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1333,10 +1384,10 @@
         <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="C17" t="s">
-        <v>255</v>
+        <v>272</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1344,10 +1395,10 @@
         <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="C18" t="s">
-        <v>258</v>
+        <v>275</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1355,10 +1406,10 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C19" t="s">
-        <v>253</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1366,10 +1417,10 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="C20" t="s">
-        <v>259</v>
+        <v>276</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1377,10 +1428,10 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="C21" t="s">
-        <v>256</v>
+        <v>273</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1388,10 +1439,10 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C22" t="s">
-        <v>260</v>
+        <v>277</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1399,10 +1450,10 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="C23" t="s">
-        <v>261</v>
+        <v>278</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1410,10 +1461,10 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="C24" t="s">
-        <v>260</v>
+        <v>277</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1421,10 +1472,10 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="C25" t="s">
-        <v>259</v>
+        <v>276</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1432,10 +1483,10 @@
         <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="C26" t="s">
-        <v>256</v>
+        <v>274</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1443,10 +1494,10 @@
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="C27" t="s">
-        <v>262</v>
+        <v>273</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1454,10 +1505,10 @@
         <v>29</v>
       </c>
       <c r="B28" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="C28" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1465,10 +1516,10 @@
         <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="C29" t="s">
-        <v>263</v>
+        <v>278</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1476,10 +1527,10 @@
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="C30" t="s">
-        <v>258</v>
+        <v>280</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1487,10 +1538,10 @@
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="C31" t="s">
-        <v>258</v>
+        <v>275</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1498,10 +1549,10 @@
         <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="C32" t="s">
-        <v>260</v>
+        <v>275</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1509,10 +1560,10 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="C33" t="s">
-        <v>264</v>
+        <v>277</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1520,10 +1571,10 @@
         <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="C34" t="s">
-        <v>265</v>
+        <v>281</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1531,10 +1582,10 @@
         <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="C35" t="s">
-        <v>252</v>
+        <v>282</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -1542,10 +1593,10 @@
         <v>37</v>
       </c>
       <c r="B36" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="C36" t="s">
-        <v>253</v>
+        <v>269</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1553,10 +1604,10 @@
         <v>38</v>
       </c>
       <c r="B37" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="C37" t="s">
-        <v>252</v>
+        <v>270</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1564,10 +1615,10 @@
         <v>39</v>
       </c>
       <c r="B38" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="C38" t="s">
-        <v>255</v>
+        <v>269</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -1575,10 +1626,10 @@
         <v>40</v>
       </c>
       <c r="B39" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="C39" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -1586,10 +1637,10 @@
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="C40" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1597,10 +1648,10 @@
         <v>42</v>
       </c>
       <c r="B41" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="C41" t="s">
-        <v>260</v>
+        <v>282</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1608,10 +1659,10 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="C42" t="s">
-        <v>261</v>
+        <v>277</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1619,10 +1670,10 @@
         <v>44</v>
       </c>
       <c r="B43" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="C43" t="s">
-        <v>261</v>
+        <v>278</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -1630,10 +1681,10 @@
         <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="C44" t="s">
-        <v>254</v>
+        <v>278</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -1641,10 +1692,10 @@
         <v>46</v>
       </c>
       <c r="B45" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="C45" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -1652,10 +1703,10 @@
         <v>47</v>
       </c>
       <c r="B46" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="C46" t="s">
-        <v>261</v>
+        <v>278</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -1663,10 +1714,10 @@
         <v>48</v>
       </c>
       <c r="B47" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="C47" t="s">
-        <v>254</v>
+        <v>278</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -1674,10 +1725,10 @@
         <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="C48" t="s">
-        <v>260</v>
+        <v>271</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -1685,10 +1736,10 @@
         <v>50</v>
       </c>
       <c r="B49" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="C49" t="s">
-        <v>263</v>
+        <v>277</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1696,10 +1747,10 @@
         <v>51</v>
       </c>
       <c r="B50" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C50" t="s">
-        <v>255</v>
+        <v>280</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -1707,10 +1758,10 @@
         <v>52</v>
       </c>
       <c r="B51" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="C51" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -1718,10 +1769,10 @@
         <v>53</v>
       </c>
       <c r="B52" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C52" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -1729,10 +1780,10 @@
         <v>54</v>
       </c>
       <c r="B53" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="C53" t="s">
-        <v>263</v>
+        <v>277</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -1740,10 +1791,10 @@
         <v>55</v>
       </c>
       <c r="B54" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="C54" t="s">
-        <v>253</v>
+        <v>269</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1751,10 +1802,10 @@
         <v>56</v>
       </c>
       <c r="B55" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C55" t="s">
-        <v>256</v>
+        <v>278</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -1762,10 +1813,10 @@
         <v>57</v>
       </c>
       <c r="B56" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="C56" t="s">
-        <v>260</v>
+        <v>280</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1773,10 +1824,10 @@
         <v>58</v>
       </c>
       <c r="B57" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="C57" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1784,10 +1835,10 @@
         <v>59</v>
       </c>
       <c r="B58" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="C58" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -1795,10 +1846,10 @@
         <v>60</v>
       </c>
       <c r="B59" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="C59" t="s">
-        <v>252</v>
+        <v>277</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1806,10 +1857,10 @@
         <v>61</v>
       </c>
       <c r="B60" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="C60" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1817,10 +1868,10 @@
         <v>62</v>
       </c>
       <c r="B61" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="C61" t="s">
-        <v>252</v>
+        <v>276</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -1828,10 +1879,10 @@
         <v>63</v>
       </c>
       <c r="B62" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="C62" t="s">
-        <v>252</v>
+        <v>269</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -1839,10 +1890,10 @@
         <v>64</v>
       </c>
       <c r="B63" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="C63" t="s">
-        <v>262</v>
+        <v>279</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -1850,10 +1901,10 @@
         <v>65</v>
       </c>
       <c r="B64" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="C64" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1861,10 +1912,10 @@
         <v>66</v>
       </c>
       <c r="B65" t="s">
-        <v>190</v>
+        <v>199</v>
       </c>
       <c r="C65" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -1872,10 +1923,10 @@
         <v>67</v>
       </c>
       <c r="B66" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="C66" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -1883,10 +1934,10 @@
         <v>68</v>
       </c>
       <c r="B67" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="C67" t="s">
-        <v>258</v>
+        <v>274</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -1894,10 +1945,10 @@
         <v>69</v>
       </c>
       <c r="B68" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="C68" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -1905,10 +1956,10 @@
         <v>70</v>
       </c>
       <c r="B69" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="C69" t="s">
-        <v>266</v>
+        <v>283</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -1916,10 +1967,7 @@
         <v>71</v>
       </c>
       <c r="B70" t="s">
-        <v>195</v>
-      </c>
-      <c r="C70" t="s">
-        <v>252</v>
+        <v>204</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -1927,10 +1975,10 @@
         <v>72</v>
       </c>
       <c r="B71" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="C71" t="s">
-        <v>252</v>
+        <v>282</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -1938,10 +1986,10 @@
         <v>73</v>
       </c>
       <c r="B72" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="C72" t="s">
-        <v>260</v>
+        <v>275</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -1949,10 +1997,10 @@
         <v>74</v>
       </c>
       <c r="B73" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="C73" t="s">
-        <v>260</v>
+        <v>277</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -1960,10 +2008,10 @@
         <v>75</v>
       </c>
       <c r="B74" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="C74" t="s">
-        <v>255</v>
+        <v>283</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -1971,10 +2019,10 @@
         <v>76</v>
       </c>
       <c r="B75" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="C75" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -1982,10 +2030,10 @@
         <v>77</v>
       </c>
       <c r="B76" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="C76" t="s">
-        <v>252</v>
+        <v>269</v>
       </c>
     </row>
     <row r="77" spans="1:3">
@@ -1993,10 +2041,10 @@
         <v>78</v>
       </c>
       <c r="B77" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="C77" t="s">
-        <v>257</v>
+        <v>277</v>
       </c>
     </row>
     <row r="78" spans="1:3">
@@ -2004,10 +2052,10 @@
         <v>79</v>
       </c>
       <c r="B78" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="C78" t="s">
-        <v>252</v>
+        <v>277</v>
       </c>
     </row>
     <row r="79" spans="1:3">
@@ -2015,10 +2063,10 @@
         <v>80</v>
       </c>
       <c r="B79" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="C79" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -2026,10 +2074,10 @@
         <v>81</v>
       </c>
       <c r="B80" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="C80" t="s">
-        <v>258</v>
+        <v>277</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -2037,10 +2085,10 @@
         <v>82</v>
       </c>
       <c r="B81" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="C81" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -2048,10 +2096,10 @@
         <v>83</v>
       </c>
       <c r="B82" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="C82" t="s">
-        <v>254</v>
+        <v>274</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -2059,10 +2107,10 @@
         <v>84</v>
       </c>
       <c r="B83" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="C83" t="s">
-        <v>252</v>
+        <v>269</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -2070,10 +2118,10 @@
         <v>85</v>
       </c>
       <c r="B84" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="C84" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -2081,10 +2129,10 @@
         <v>86</v>
       </c>
       <c r="B85" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="C85" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -2092,10 +2140,10 @@
         <v>87</v>
       </c>
       <c r="B86" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="C86" t="s">
-        <v>256</v>
+        <v>275</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -2103,7 +2151,10 @@
         <v>88</v>
       </c>
       <c r="B87" t="s">
-        <v>212</v>
+        <v>221</v>
+      </c>
+      <c r="C87" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -2111,10 +2162,10 @@
         <v>89</v>
       </c>
       <c r="B88" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="C88" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -2122,10 +2173,10 @@
         <v>90</v>
       </c>
       <c r="B89" t="s">
-        <v>214</v>
+        <v>223</v>
       </c>
       <c r="C89" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -2133,10 +2184,10 @@
         <v>91</v>
       </c>
       <c r="B90" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
       <c r="C90" t="s">
-        <v>252</v>
+        <v>277</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -2144,10 +2195,10 @@
         <v>92</v>
       </c>
       <c r="B91" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="C91" t="s">
-        <v>252</v>
+        <v>277</v>
       </c>
     </row>
     <row r="92" spans="1:3">
@@ -2155,10 +2206,10 @@
         <v>93</v>
       </c>
       <c r="B92" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="C92" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -2166,10 +2217,10 @@
         <v>94</v>
       </c>
       <c r="B93" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="C93" t="s">
-        <v>262</v>
+        <v>277</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -2177,10 +2228,10 @@
         <v>95</v>
       </c>
       <c r="B94" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="C94" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -2188,10 +2239,10 @@
         <v>96</v>
       </c>
       <c r="B95" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="C95" t="s">
-        <v>262</v>
+        <v>284</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -2199,10 +2250,10 @@
         <v>97</v>
       </c>
       <c r="B96" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
       <c r="C96" t="s">
-        <v>252</v>
+        <v>277</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -2210,10 +2261,10 @@
         <v>98</v>
       </c>
       <c r="B97" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="C97" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -2221,10 +2272,10 @@
         <v>99</v>
       </c>
       <c r="B98" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="C98" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
     </row>
     <row r="99" spans="1:3">
@@ -2232,10 +2283,10 @@
         <v>100</v>
       </c>
       <c r="B99" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="C99" t="s">
-        <v>261</v>
+        <v>274</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -2243,10 +2294,10 @@
         <v>101</v>
       </c>
       <c r="B100" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="C100" t="s">
-        <v>260</v>
+        <v>279</v>
       </c>
     </row>
     <row r="101" spans="1:3">
@@ -2254,10 +2305,10 @@
         <v>102</v>
       </c>
       <c r="B101" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="C101" t="s">
-        <v>256</v>
+        <v>277</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -2265,10 +2316,10 @@
         <v>103</v>
       </c>
       <c r="B102" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="C102" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -2276,10 +2327,10 @@
         <v>104</v>
       </c>
       <c r="B103" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C103" t="s">
-        <v>252</v>
+        <v>269</v>
       </c>
     </row>
     <row r="104" spans="1:3">
@@ -2287,10 +2338,10 @@
         <v>105</v>
       </c>
       <c r="B104" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="C104" t="s">
-        <v>253</v>
+        <v>279</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -2298,10 +2349,10 @@
         <v>106</v>
       </c>
       <c r="B105" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="C105" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
     </row>
     <row r="106" spans="1:3">
@@ -2309,10 +2360,10 @@
         <v>107</v>
       </c>
       <c r="B106" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="C106" t="s">
-        <v>257</v>
+        <v>278</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -2320,10 +2371,10 @@
         <v>108</v>
       </c>
       <c r="B107" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="C107" t="s">
-        <v>252</v>
+        <v>277</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -2331,10 +2382,10 @@
         <v>109</v>
       </c>
       <c r="B108" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="C108" t="s">
-        <v>257</v>
+        <v>273</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -2342,10 +2393,10 @@
         <v>110</v>
       </c>
       <c r="B109" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="C109" t="s">
-        <v>255</v>
+        <v>283</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -2353,10 +2404,10 @@
         <v>111</v>
       </c>
       <c r="B110" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="C110" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="111" spans="1:3">
@@ -2364,10 +2415,10 @@
         <v>112</v>
       </c>
       <c r="B111" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="C111" t="s">
-        <v>255</v>
+        <v>270</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -2375,10 +2426,10 @@
         <v>113</v>
       </c>
       <c r="B112" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="C112" t="s">
-        <v>255</v>
+        <v>278</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -2386,10 +2437,10 @@
         <v>114</v>
       </c>
       <c r="B113" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="C113" t="s">
-        <v>253</v>
+        <v>274</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -2397,10 +2448,10 @@
         <v>115</v>
       </c>
       <c r="B114" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="C114" t="s">
-        <v>254</v>
+        <v>269</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -2408,10 +2459,10 @@
         <v>116</v>
       </c>
       <c r="B115" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="C115" t="s">
-        <v>263</v>
+        <v>274</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -2419,10 +2470,10 @@
         <v>117</v>
       </c>
       <c r="B116" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="C116" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="117" spans="1:3">
@@ -2430,10 +2481,10 @@
         <v>118</v>
       </c>
       <c r="B117" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="C117" t="s">
-        <v>266</v>
+        <v>282</v>
       </c>
     </row>
     <row r="118" spans="1:3">
@@ -2441,10 +2492,10 @@
         <v>119</v>
       </c>
       <c r="B118" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="C118" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -2452,10 +2503,10 @@
         <v>120</v>
       </c>
       <c r="B119" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="C119" t="s">
-        <v>256</v>
+        <v>282</v>
       </c>
     </row>
     <row r="120" spans="1:3">
@@ -2463,10 +2514,10 @@
         <v>121</v>
       </c>
       <c r="B120" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="C120" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
     </row>
     <row r="121" spans="1:3">
@@ -2474,10 +2525,10 @@
         <v>122</v>
       </c>
       <c r="B121" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="C121" t="s">
-        <v>254</v>
+        <v>270</v>
       </c>
     </row>
     <row r="122" spans="1:3">
@@ -2485,10 +2536,10 @@
         <v>123</v>
       </c>
       <c r="B122" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="C122" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
     </row>
     <row r="123" spans="1:3">
@@ -2496,10 +2547,10 @@
         <v>124</v>
       </c>
       <c r="B123" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="C123" t="s">
-        <v>253</v>
+        <v>280</v>
       </c>
     </row>
     <row r="124" spans="1:3">
@@ -2507,10 +2558,10 @@
         <v>125</v>
       </c>
       <c r="B124" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="C124" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="125" spans="1:3">
@@ -2518,10 +2569,10 @@
         <v>126</v>
       </c>
       <c r="B125" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="C125" t="s">
-        <v>260</v>
+        <v>283</v>
       </c>
     </row>
     <row r="126" spans="1:3">
@@ -2529,10 +2580,98 @@
         <v>127</v>
       </c>
       <c r="B126" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="C126" t="s">
-        <v>252</v>
+        <v>279</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3">
+      <c r="A127" t="s">
+        <v>128</v>
+      </c>
+      <c r="B127" t="s">
+        <v>261</v>
+      </c>
+      <c r="C127" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3">
+      <c r="A128" t="s">
+        <v>129</v>
+      </c>
+      <c r="B128" t="s">
+        <v>262</v>
+      </c>
+      <c r="C128" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3">
+      <c r="A129" t="s">
+        <v>130</v>
+      </c>
+      <c r="B129" t="s">
+        <v>263</v>
+      </c>
+      <c r="C129" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3">
+      <c r="A130" t="s">
+        <v>131</v>
+      </c>
+      <c r="B130" t="s">
+        <v>264</v>
+      </c>
+      <c r="C130" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3">
+      <c r="A131" t="s">
+        <v>132</v>
+      </c>
+      <c r="B131" t="s">
+        <v>265</v>
+      </c>
+      <c r="C131" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3">
+      <c r="A132" t="s">
+        <v>133</v>
+      </c>
+      <c r="B132" t="s">
+        <v>266</v>
+      </c>
+      <c r="C132" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3">
+      <c r="A133" t="s">
+        <v>134</v>
+      </c>
+      <c r="B133" t="s">
+        <v>267</v>
+      </c>
+      <c r="C133" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3">
+      <c r="A134" t="s">
+        <v>135</v>
+      </c>
+      <c r="B134" t="s">
+        <v>268</v>
+      </c>
+      <c r="C134" t="s">
+        <v>269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update student fee registry
This commit adds new student records and codes to the registry, updates several existing fee entries, and corrects totals and balances in the first-term student dataset. It also refreshes the Excel fee and parent-code files to match the latest academic-year data.
</commit_message>
<xml_diff>
--- a/parent_codes.xlsx
+++ b/parent_codes.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="294">
   <si>
     <t>Code</t>
   </si>
@@ -142,6 +142,9 @@
     <t>AKIGAB1034</t>
   </si>
   <si>
+    <t>AKPFRA1138</t>
+  </si>
+  <si>
     <t>ALAADE1036</t>
   </si>
   <si>
@@ -274,6 +277,9 @@
     <t>MORPRI1134</t>
   </si>
   <si>
+    <t>MORTES1139</t>
+  </si>
+  <si>
     <t>MOSHEP1074</t>
   </si>
   <si>
@@ -307,6 +313,9 @@
     <t>OKEJUM1081</t>
   </si>
   <si>
+    <t>OLAABD1140</t>
+  </si>
+  <si>
     <t>OLAADE1086</t>
   </si>
   <si>
@@ -355,6 +364,9 @@
     <t>OLUTEM1098</t>
   </si>
   <si>
+    <t>ONIAAR1141</t>
+  </si>
+  <si>
     <t>ONOMIR1099</t>
   </si>
   <si>
@@ -541,6 +553,9 @@
     <t>AKINDURO GABRIELLA OLUWAFIREWAMIRI</t>
   </si>
   <si>
+    <t>AKPAN FRANCIS</t>
+  </si>
+  <si>
     <t>ALABI ADEKUNLE</t>
   </si>
   <si>
@@ -673,6 +688,9 @@
     <t>MORADEYO PRISCILLA OLUWADARASIMI</t>
   </si>
   <si>
+    <t>MORAKINYO TESTIMONY AYANFE</t>
+  </si>
+  <si>
     <t>MOSES HEPHZIBAH TOLUWALASE</t>
   </si>
   <si>
@@ -706,6 +724,9 @@
     <t>OKERINDE JUMAIN BOLUWATIFE</t>
   </si>
   <si>
+    <t>OLADOSU ABDULLAHI OLUWASEYI</t>
+  </si>
+  <si>
     <t>OLALEMI ADEMIDE SAMUEL</t>
   </si>
   <si>
@@ -754,6 +775,9 @@
     <t>OLUWASHOLA TEMILOLUWA ELIZABETH</t>
   </si>
   <si>
+    <t>ONI AARON OLUWADEMILADE</t>
+  </si>
+  <si>
     <t>ONOJA MIRACLE</t>
   </si>
   <si>
@@ -866,6 +890,9 @@
   </si>
   <si>
     <t>PRIMARY 4</t>
+  </si>
+  <si>
+    <t>PRINARY 2</t>
   </si>
   <si>
     <t>SENIOR SECONDARY SCHOOL 3</t>
@@ -1200,7 +1227,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1219,10 +1246,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C2" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1230,10 +1257,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C3" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1241,10 +1268,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C4" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1252,10 +1279,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C5" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1263,10 +1290,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C6" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1274,10 +1301,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C7" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1285,10 +1312,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C8" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1296,10 +1323,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C9" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1307,10 +1334,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C10" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1318,10 +1345,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C11" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1329,10 +1356,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C12" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1340,10 +1367,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C13" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1351,10 +1378,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C14" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1362,10 +1389,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C15" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1373,10 +1400,10 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C16" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1384,10 +1411,10 @@
         <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C17" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1395,10 +1422,10 @@
         <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C18" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1406,10 +1433,10 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C19" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1417,10 +1444,10 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C20" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1428,10 +1455,10 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C21" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1439,10 +1466,10 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C22" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1450,10 +1477,10 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C23" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1461,10 +1488,10 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C24" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1472,10 +1499,10 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C25" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1483,10 +1510,10 @@
         <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C26" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1494,10 +1521,10 @@
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C27" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1505,10 +1532,10 @@
         <v>29</v>
       </c>
       <c r="B28" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C28" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1516,10 +1543,10 @@
         <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C29" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1527,10 +1554,10 @@
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C30" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1538,10 +1565,10 @@
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C31" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1549,10 +1576,10 @@
         <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C32" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1560,10 +1587,10 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C33" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1571,10 +1598,10 @@
         <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C34" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1582,10 +1609,10 @@
         <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="C35" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -1593,10 +1620,10 @@
         <v>37</v>
       </c>
       <c r="B36" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C36" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1604,10 +1631,10 @@
         <v>38</v>
       </c>
       <c r="B37" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="C37" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1615,10 +1642,10 @@
         <v>39</v>
       </c>
       <c r="B38" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C38" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -1626,10 +1653,10 @@
         <v>40</v>
       </c>
       <c r="B39" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C39" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -1637,10 +1664,10 @@
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C40" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1648,10 +1675,10 @@
         <v>42</v>
       </c>
       <c r="B41" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C41" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1659,10 +1686,10 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C42" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1670,10 +1697,10 @@
         <v>44</v>
       </c>
       <c r="B43" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C43" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -1681,10 +1708,10 @@
         <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C44" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -1692,10 +1719,10 @@
         <v>46</v>
       </c>
       <c r="B45" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C45" t="s">
-        <v>271</v>
+        <v>286</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -1703,10 +1730,10 @@
         <v>47</v>
       </c>
       <c r="B46" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C46" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -1714,10 +1741,10 @@
         <v>48</v>
       </c>
       <c r="B47" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C47" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -1725,10 +1752,10 @@
         <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C48" t="s">
-        <v>271</v>
+        <v>286</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -1736,10 +1763,10 @@
         <v>50</v>
       </c>
       <c r="B49" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C49" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1747,10 +1774,10 @@
         <v>51</v>
       </c>
       <c r="B50" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C50" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -1758,10 +1785,10 @@
         <v>52</v>
       </c>
       <c r="B51" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C51" t="s">
-        <v>272</v>
+        <v>288</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -1769,10 +1796,10 @@
         <v>53</v>
       </c>
       <c r="B52" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C52" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -1780,10 +1807,10 @@
         <v>54</v>
       </c>
       <c r="B53" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C53" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -1791,10 +1818,10 @@
         <v>55</v>
       </c>
       <c r="B54" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C54" t="s">
-        <v>269</v>
+        <v>285</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1802,10 +1829,10 @@
         <v>56</v>
       </c>
       <c r="B55" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C55" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -1813,10 +1840,10 @@
         <v>57</v>
       </c>
       <c r="B56" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C56" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1824,10 +1851,10 @@
         <v>58</v>
       </c>
       <c r="B57" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C57" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1835,10 +1862,10 @@
         <v>59</v>
       </c>
       <c r="B58" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="C58" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -1846,10 +1873,10 @@
         <v>60</v>
       </c>
       <c r="B59" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C59" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1857,10 +1884,10 @@
         <v>61</v>
       </c>
       <c r="B60" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C60" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1868,10 +1895,10 @@
         <v>62</v>
       </c>
       <c r="B61" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C61" t="s">
-        <v>276</v>
+        <v>286</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -1879,10 +1906,10 @@
         <v>63</v>
       </c>
       <c r="B62" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C62" t="s">
-        <v>269</v>
+        <v>284</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -1890,10 +1917,10 @@
         <v>64</v>
       </c>
       <c r="B63" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C63" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -1901,10 +1928,10 @@
         <v>65</v>
       </c>
       <c r="B64" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C64" t="s">
-        <v>269</v>
+        <v>287</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1912,10 +1939,10 @@
         <v>66</v>
       </c>
       <c r="B65" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C65" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -1923,10 +1950,10 @@
         <v>67</v>
       </c>
       <c r="B66" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C66" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -1934,10 +1961,10 @@
         <v>68</v>
       </c>
       <c r="B67" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C67" t="s">
-        <v>274</v>
+        <v>287</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -1945,10 +1972,10 @@
         <v>69</v>
       </c>
       <c r="B68" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C68" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -1956,10 +1983,10 @@
         <v>70</v>
       </c>
       <c r="B69" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C69" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -1967,7 +1994,10 @@
         <v>71</v>
       </c>
       <c r="B70" t="s">
-        <v>204</v>
+        <v>208</v>
+      </c>
+      <c r="C70" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -1975,10 +2005,10 @@
         <v>72</v>
       </c>
       <c r="B71" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C71" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -1986,10 +2016,10 @@
         <v>73</v>
       </c>
       <c r="B72" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C72" t="s">
-        <v>275</v>
+        <v>290</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -1997,10 +2027,10 @@
         <v>74</v>
       </c>
       <c r="B73" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C73" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -2008,10 +2038,10 @@
         <v>75</v>
       </c>
       <c r="B74" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="C74" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -2019,10 +2049,10 @@
         <v>76</v>
       </c>
       <c r="B75" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C75" t="s">
-        <v>269</v>
+        <v>291</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -2030,10 +2060,10 @@
         <v>77</v>
       </c>
       <c r="B76" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C76" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="77" spans="1:3">
@@ -2041,7 +2071,7 @@
         <v>78</v>
       </c>
       <c r="B77" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C77" t="s">
         <v>277</v>
@@ -2052,10 +2082,10 @@
         <v>79</v>
       </c>
       <c r="B78" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="C78" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="79" spans="1:3">
@@ -2063,10 +2093,10 @@
         <v>80</v>
       </c>
       <c r="B79" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C79" t="s">
-        <v>272</v>
+        <v>285</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -2074,10 +2104,10 @@
         <v>81</v>
       </c>
       <c r="B80" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C80" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -2085,10 +2115,10 @@
         <v>82</v>
       </c>
       <c r="B81" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C81" t="s">
-        <v>269</v>
+        <v>285</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -2096,10 +2126,10 @@
         <v>83</v>
       </c>
       <c r="B82" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C82" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -2107,10 +2137,10 @@
         <v>84</v>
       </c>
       <c r="B83" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C83" t="s">
-        <v>269</v>
+        <v>282</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -2118,10 +2148,10 @@
         <v>85</v>
       </c>
       <c r="B84" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C84" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -2129,10 +2159,10 @@
         <v>86</v>
       </c>
       <c r="B85" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C85" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -2140,10 +2170,10 @@
         <v>87</v>
       </c>
       <c r="B86" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="C86" t="s">
-        <v>275</v>
+        <v>288</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -2151,10 +2181,10 @@
         <v>88</v>
       </c>
       <c r="B87" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C87" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -2162,10 +2192,10 @@
         <v>89</v>
       </c>
       <c r="B88" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C88" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -2173,10 +2203,10 @@
         <v>90</v>
       </c>
       <c r="B89" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="C89" t="s">
-        <v>269</v>
+        <v>282</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -2184,10 +2214,10 @@
         <v>91</v>
       </c>
       <c r="B90" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C90" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -2195,7 +2225,7 @@
         <v>92</v>
       </c>
       <c r="B91" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C91" t="s">
         <v>277</v>
@@ -2206,10 +2236,10 @@
         <v>93</v>
       </c>
       <c r="B92" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="C92" t="s">
-        <v>269</v>
+        <v>285</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -2217,10 +2247,10 @@
         <v>94</v>
       </c>
       <c r="B93" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C93" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -2228,10 +2258,10 @@
         <v>95</v>
       </c>
       <c r="B94" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="C94" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -2239,10 +2269,10 @@
         <v>96</v>
       </c>
       <c r="B95" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C95" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -2250,10 +2280,10 @@
         <v>97</v>
       </c>
       <c r="B96" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C96" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -2261,10 +2291,10 @@
         <v>98</v>
       </c>
       <c r="B97" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="C97" t="s">
-        <v>269</v>
+        <v>293</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -2272,10 +2302,10 @@
         <v>99</v>
       </c>
       <c r="B98" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="C98" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="99" spans="1:3">
@@ -2283,10 +2313,10 @@
         <v>100</v>
       </c>
       <c r="B99" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C99" t="s">
-        <v>274</v>
+        <v>285</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -2294,10 +2324,10 @@
         <v>101</v>
       </c>
       <c r="B100" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C100" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="101" spans="1:3">
@@ -2305,7 +2335,7 @@
         <v>102</v>
       </c>
       <c r="B101" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="C101" t="s">
         <v>277</v>
@@ -2316,10 +2346,10 @@
         <v>103</v>
       </c>
       <c r="B102" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C102" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -2327,10 +2357,10 @@
         <v>104</v>
       </c>
       <c r="B103" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C103" t="s">
-        <v>269</v>
+        <v>287</v>
       </c>
     </row>
     <row r="104" spans="1:3">
@@ -2338,10 +2368,10 @@
         <v>105</v>
       </c>
       <c r="B104" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C104" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -2349,10 +2379,10 @@
         <v>106</v>
       </c>
       <c r="B105" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C105" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
     </row>
     <row r="106" spans="1:3">
@@ -2360,10 +2390,10 @@
         <v>107</v>
       </c>
       <c r="B106" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C106" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -2371,10 +2401,10 @@
         <v>108</v>
       </c>
       <c r="B107" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C107" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -2382,10 +2412,10 @@
         <v>109</v>
       </c>
       <c r="B108" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="C108" t="s">
-        <v>273</v>
+        <v>287</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -2393,10 +2423,10 @@
         <v>110</v>
       </c>
       <c r="B109" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C109" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -2404,10 +2434,10 @@
         <v>111</v>
       </c>
       <c r="B110" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C110" t="s">
-        <v>269</v>
+        <v>285</v>
       </c>
     </row>
     <row r="111" spans="1:3">
@@ -2415,10 +2445,10 @@
         <v>112</v>
       </c>
       <c r="B111" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="C111" t="s">
-        <v>270</v>
+        <v>281</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -2426,10 +2456,10 @@
         <v>113</v>
       </c>
       <c r="B112" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C112" t="s">
-        <v>278</v>
+        <v>291</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -2437,10 +2467,10 @@
         <v>114</v>
       </c>
       <c r="B113" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="C113" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -2448,10 +2478,10 @@
         <v>115</v>
       </c>
       <c r="B114" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C114" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -2459,10 +2489,10 @@
         <v>116</v>
       </c>
       <c r="B115" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="C115" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
     </row>
     <row r="116" spans="1:3">
@@ -2470,10 +2500,10 @@
         <v>117</v>
       </c>
       <c r="B116" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C116" t="s">
-        <v>272</v>
+        <v>286</v>
       </c>
     </row>
     <row r="117" spans="1:3">
@@ -2481,7 +2511,7 @@
         <v>118</v>
       </c>
       <c r="B117" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="C117" t="s">
         <v>282</v>
@@ -2492,10 +2522,10 @@
         <v>119</v>
       </c>
       <c r="B118" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="C118" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -2503,7 +2533,7 @@
         <v>120</v>
       </c>
       <c r="B119" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="C119" t="s">
         <v>282</v>
@@ -2514,10 +2544,10 @@
         <v>121</v>
       </c>
       <c r="B120" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="C120" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
     </row>
     <row r="121" spans="1:3">
@@ -2525,10 +2555,10 @@
         <v>122</v>
       </c>
       <c r="B121" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="C121" t="s">
-        <v>270</v>
+        <v>290</v>
       </c>
     </row>
     <row r="122" spans="1:3">
@@ -2536,10 +2566,10 @@
         <v>123</v>
       </c>
       <c r="B122" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="C122" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
     </row>
     <row r="123" spans="1:3">
@@ -2547,10 +2577,10 @@
         <v>124</v>
       </c>
       <c r="B123" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="C123" t="s">
-        <v>280</v>
+        <v>290</v>
       </c>
     </row>
     <row r="124" spans="1:3">
@@ -2558,10 +2588,10 @@
         <v>125</v>
       </c>
       <c r="B124" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C124" t="s">
-        <v>269</v>
+        <v>280</v>
       </c>
     </row>
     <row r="125" spans="1:3">
@@ -2569,10 +2599,10 @@
         <v>126</v>
       </c>
       <c r="B125" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="C125" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="126" spans="1:3">
@@ -2580,7 +2610,7 @@
         <v>127</v>
       </c>
       <c r="B126" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="C126" t="s">
         <v>279</v>
@@ -2591,10 +2621,10 @@
         <v>128</v>
       </c>
       <c r="B127" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="C127" t="s">
-        <v>273</v>
+        <v>288</v>
       </c>
     </row>
     <row r="128" spans="1:3">
@@ -2602,7 +2632,7 @@
         <v>129</v>
       </c>
       <c r="B128" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C128" t="s">
         <v>277</v>
@@ -2613,10 +2643,10 @@
         <v>130</v>
       </c>
       <c r="B129" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C129" t="s">
-        <v>271</v>
+        <v>291</v>
       </c>
     </row>
     <row r="130" spans="1:3">
@@ -2624,10 +2654,10 @@
         <v>131</v>
       </c>
       <c r="B130" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C130" t="s">
-        <v>278</v>
+        <v>287</v>
       </c>
     </row>
     <row r="131" spans="1:3">
@@ -2635,10 +2665,10 @@
         <v>132</v>
       </c>
       <c r="B131" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C131" t="s">
-        <v>270</v>
+        <v>281</v>
       </c>
     </row>
     <row r="132" spans="1:3">
@@ -2646,10 +2676,10 @@
         <v>133</v>
       </c>
       <c r="B132" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="C132" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
     </row>
     <row r="133" spans="1:3">
@@ -2657,10 +2687,10 @@
         <v>134</v>
       </c>
       <c r="B133" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C133" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="134" spans="1:3">
@@ -2668,10 +2698,54 @@
         <v>135</v>
       </c>
       <c r="B134" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C134" t="s">
-        <v>269</v>
+        <v>286</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3">
+      <c r="A135" t="s">
+        <v>136</v>
+      </c>
+      <c r="B135" t="s">
+        <v>273</v>
+      </c>
+      <c r="C135" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3">
+      <c r="A136" t="s">
+        <v>137</v>
+      </c>
+      <c r="B136" t="s">
+        <v>274</v>
+      </c>
+      <c r="C136" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3">
+      <c r="A137" t="s">
+        <v>138</v>
+      </c>
+      <c r="B137" t="s">
+        <v>275</v>
+      </c>
+      <c r="C137" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3">
+      <c r="A138" t="s">
+        <v>139</v>
+      </c>
+      <c r="B138" t="s">
+        <v>276</v>
+      </c>
+      <c r="C138" t="s">
+        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update fee data and student codes
Added the registry entry for NURUDEEN ABU-BAKIR (NURABU1142) and updated fee records for multiple students in the first-term dataset. This includes corrected total fees, payments, balances, and synchronized changes across the Excel files and student registry.
</commit_message>
<xml_diff>
--- a/parent_codes.xlsx
+++ b/parent_codes.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="295">
   <si>
     <t>Code</t>
   </si>
@@ -295,6 +295,9 @@
     <t>NELHAR1078</t>
   </si>
   <si>
+    <t>NURABU1142</t>
+  </si>
+  <si>
     <t>OBEKEH1080</t>
   </si>
   <si>
@@ -704,6 +707,9 @@
   </si>
   <si>
     <t>NELSON HARRY EMMANUEL OBALOLUWA</t>
+  </si>
+  <si>
+    <t>NURUDEEN ABU-BAKIR</t>
   </si>
   <si>
     <t>OBEY KEHINDE AYOLEYI</t>
@@ -1224,7 +1230,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1243,10 +1249,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C2" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1254,10 +1260,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1265,10 +1271,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C4" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1276,10 +1282,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C5" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1287,10 +1293,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C6" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1298,10 +1304,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C7" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1309,10 +1315,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C8" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1320,10 +1326,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C9" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1331,10 +1337,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C10" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1342,10 +1348,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C11" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1353,10 +1359,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C12" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1364,10 +1370,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C13" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1375,10 +1381,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C14" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1386,10 +1392,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C15" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1397,10 +1403,10 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C16" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1408,10 +1414,10 @@
         <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C17" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1419,10 +1425,10 @@
         <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C18" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1430,10 +1436,10 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C19" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1441,10 +1447,10 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C20" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1452,10 +1458,10 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C21" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1463,10 +1469,10 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C22" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1474,10 +1480,10 @@
         <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C23" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1485,10 +1491,10 @@
         <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C24" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1496,10 +1502,10 @@
         <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C25" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1507,10 +1513,10 @@
         <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C26" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1518,10 +1524,10 @@
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C27" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1529,10 +1535,10 @@
         <v>29</v>
       </c>
       <c r="B28" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C28" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -1540,10 +1546,10 @@
         <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C29" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1551,10 +1557,10 @@
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C30" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -1562,10 +1568,10 @@
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C31" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1573,10 +1579,10 @@
         <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C32" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1584,10 +1590,10 @@
         <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C33" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1595,10 +1601,10 @@
         <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C34" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -1606,10 +1612,10 @@
         <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C35" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -1617,10 +1623,10 @@
         <v>37</v>
       </c>
       <c r="B36" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C36" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -1628,10 +1634,10 @@
         <v>38</v>
       </c>
       <c r="B37" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C37" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -1639,10 +1645,10 @@
         <v>39</v>
       </c>
       <c r="B38" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C38" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="39" spans="1:3">
@@ -1650,10 +1656,10 @@
         <v>40</v>
       </c>
       <c r="B39" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C39" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -1661,10 +1667,10 @@
         <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C40" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="41" spans="1:3">
@@ -1672,10 +1678,10 @@
         <v>42</v>
       </c>
       <c r="B41" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C41" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="42" spans="1:3">
@@ -1683,10 +1689,10 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C42" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -1694,10 +1700,10 @@
         <v>44</v>
       </c>
       <c r="B43" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C43" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -1705,10 +1711,10 @@
         <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C44" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -1716,10 +1722,10 @@
         <v>46</v>
       </c>
       <c r="B45" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C45" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="46" spans="1:3">
@@ -1727,10 +1733,10 @@
         <v>47</v>
       </c>
       <c r="B46" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C46" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -1738,10 +1744,10 @@
         <v>48</v>
       </c>
       <c r="B47" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C47" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="48" spans="1:3">
@@ -1749,10 +1755,10 @@
         <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C48" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="49" spans="1:3">
@@ -1760,10 +1766,10 @@
         <v>50</v>
       </c>
       <c r="B49" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C49" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="50" spans="1:3">
@@ -1771,10 +1777,10 @@
         <v>51</v>
       </c>
       <c r="B50" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C50" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="51" spans="1:3">
@@ -1782,10 +1788,10 @@
         <v>52</v>
       </c>
       <c r="B51" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C51" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -1793,10 +1799,10 @@
         <v>53</v>
       </c>
       <c r="B52" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C52" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="53" spans="1:3">
@@ -1804,10 +1810,10 @@
         <v>54</v>
       </c>
       <c r="B53" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C53" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="54" spans="1:3">
@@ -1815,10 +1821,10 @@
         <v>55</v>
       </c>
       <c r="B54" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C54" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="55" spans="1:3">
@@ -1826,10 +1832,10 @@
         <v>56</v>
       </c>
       <c r="B55" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C55" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -1837,10 +1843,10 @@
         <v>57</v>
       </c>
       <c r="B56" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C56" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -1848,10 +1854,10 @@
         <v>58</v>
       </c>
       <c r="B57" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C57" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -1859,10 +1865,10 @@
         <v>59</v>
       </c>
       <c r="B58" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C58" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -1870,10 +1876,10 @@
         <v>60</v>
       </c>
       <c r="B59" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C59" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -1881,10 +1887,10 @@
         <v>61</v>
       </c>
       <c r="B60" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C60" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -1892,10 +1898,10 @@
         <v>62</v>
       </c>
       <c r="B61" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C61" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -1903,10 +1909,10 @@
         <v>63</v>
       </c>
       <c r="B62" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C62" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -1914,10 +1920,10 @@
         <v>64</v>
       </c>
       <c r="B63" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C63" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -1925,10 +1931,10 @@
         <v>65</v>
       </c>
       <c r="B64" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C64" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -1936,10 +1942,10 @@
         <v>66</v>
       </c>
       <c r="B65" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C65" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="66" spans="1:3">
@@ -1947,10 +1953,10 @@
         <v>67</v>
       </c>
       <c r="B66" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C66" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -1958,10 +1964,10 @@
         <v>68</v>
       </c>
       <c r="B67" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C67" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -1969,10 +1975,10 @@
         <v>69</v>
       </c>
       <c r="B68" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C68" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -1980,10 +1986,10 @@
         <v>70</v>
       </c>
       <c r="B69" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C69" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="70" spans="1:3">
@@ -1991,10 +1997,10 @@
         <v>71</v>
       </c>
       <c r="B70" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C70" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -2002,10 +2008,10 @@
         <v>72</v>
       </c>
       <c r="B71" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C71" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -2013,10 +2019,10 @@
         <v>73</v>
       </c>
       <c r="B72" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C72" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -2024,10 +2030,10 @@
         <v>74</v>
       </c>
       <c r="B73" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C73" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -2035,10 +2041,10 @@
         <v>75</v>
       </c>
       <c r="B74" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C74" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -2046,10 +2052,10 @@
         <v>76</v>
       </c>
       <c r="B75" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C75" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -2057,10 +2063,10 @@
         <v>77</v>
       </c>
       <c r="B76" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C76" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="77" spans="1:3">
@@ -2068,10 +2074,10 @@
         <v>78</v>
       </c>
       <c r="B77" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C77" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="78" spans="1:3">
@@ -2079,10 +2085,10 @@
         <v>79</v>
       </c>
       <c r="B78" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C78" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="79" spans="1:3">
@@ -2090,10 +2096,10 @@
         <v>80</v>
       </c>
       <c r="B79" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C79" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -2101,10 +2107,10 @@
         <v>81</v>
       </c>
       <c r="B80" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C80" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -2112,10 +2118,10 @@
         <v>82</v>
       </c>
       <c r="B81" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C81" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -2123,10 +2129,10 @@
         <v>83</v>
       </c>
       <c r="B82" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C82" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="83" spans="1:3">
@@ -2134,10 +2140,10 @@
         <v>84</v>
       </c>
       <c r="B83" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C83" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -2145,10 +2151,10 @@
         <v>85</v>
       </c>
       <c r="B84" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C84" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="85" spans="1:3">
@@ -2156,10 +2162,10 @@
         <v>86</v>
       </c>
       <c r="B85" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C85" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -2167,10 +2173,10 @@
         <v>87</v>
       </c>
       <c r="B86" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C86" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -2178,10 +2184,10 @@
         <v>88</v>
       </c>
       <c r="B87" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C87" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -2189,10 +2195,10 @@
         <v>89</v>
       </c>
       <c r="B88" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C88" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -2200,10 +2206,10 @@
         <v>90</v>
       </c>
       <c r="B89" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C89" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -2211,10 +2217,10 @@
         <v>91</v>
       </c>
       <c r="B90" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C90" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -2222,10 +2228,10 @@
         <v>92</v>
       </c>
       <c r="B91" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C91" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="92" spans="1:3">
@@ -2233,10 +2239,10 @@
         <v>93</v>
       </c>
       <c r="B92" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C92" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -2244,10 +2250,10 @@
         <v>94</v>
       </c>
       <c r="B93" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C93" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -2255,10 +2261,10 @@
         <v>95</v>
       </c>
       <c r="B94" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C94" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -2266,10 +2272,10 @@
         <v>96</v>
       </c>
       <c r="B95" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C95" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -2277,10 +2283,10 @@
         <v>97</v>
       </c>
       <c r="B96" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C96" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -2288,10 +2294,10 @@
         <v>98</v>
       </c>
       <c r="B97" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C97" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -2299,10 +2305,10 @@
         <v>99</v>
       </c>
       <c r="B98" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C98" t="s">
-        <v>277</v>
+        <v>294</v>
       </c>
     </row>
     <row r="99" spans="1:3">
@@ -2310,10 +2316,10 @@
         <v>100</v>
       </c>
       <c r="B99" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C99" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -2321,10 +2327,10 @@
         <v>101</v>
       </c>
       <c r="B100" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C100" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
     </row>
     <row r="101" spans="1:3">
@@ -2332,10 +2338,10 @@
         <v>102</v>
       </c>
       <c r="B101" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C101" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -2343,10 +2349,10 @@
         <v>103</v>
       </c>
       <c r="B102" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C102" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -2354,10 +2360,10 @@
         <v>104</v>
       </c>
       <c r="B103" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C103" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="104" spans="1:3">
@@ -2365,10 +2371,10 @@
         <v>105</v>
       </c>
       <c r="B104" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C104" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -2376,7 +2382,7 @@
         <v>106</v>
       </c>
       <c r="B105" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C105" t="s">
         <v>287</v>
@@ -2387,10 +2393,10 @@
         <v>107</v>
       </c>
       <c r="B106" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C106" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -2398,10 +2404,10 @@
         <v>108</v>
       </c>
       <c r="B107" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C107" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -2409,10 +2415,10 @@
         <v>109</v>
       </c>
       <c r="B108" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C108" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -2420,10 +2426,10 @@
         <v>110</v>
       </c>
       <c r="B109" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C109" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -2431,10 +2437,10 @@
         <v>111</v>
       </c>
       <c r="B110" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C110" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="111" spans="1:3">
@@ -2442,10 +2448,10 @@
         <v>112</v>
       </c>
       <c r="B111" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C111" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -2453,10 +2459,10 @@
         <v>113</v>
       </c>
       <c r="B112" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C112" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
     </row>
     <row r="113" spans="1:3">
@@ -2464,10 +2470,10 @@
         <v>114</v>
       </c>
       <c r="B113" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C113" t="s">
-        <v>277</v>
+        <v>293</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -2475,10 +2481,10 @@
         <v>115</v>
       </c>
       <c r="B114" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C114" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -2486,7 +2492,7 @@
         <v>116</v>
       </c>
       <c r="B115" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C115" t="s">
         <v>280</v>
@@ -2497,10 +2503,10 @@
         <v>117</v>
       </c>
       <c r="B116" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C116" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
     </row>
     <row r="117" spans="1:3">
@@ -2508,10 +2514,10 @@
         <v>118</v>
       </c>
       <c r="B117" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C117" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
     </row>
     <row r="118" spans="1:3">
@@ -2519,10 +2525,10 @@
         <v>119</v>
       </c>
       <c r="B118" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C118" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -2530,10 +2536,10 @@
         <v>120</v>
       </c>
       <c r="B119" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C119" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="120" spans="1:3">
@@ -2541,10 +2547,10 @@
         <v>121</v>
       </c>
       <c r="B120" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C120" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
     </row>
     <row r="121" spans="1:3">
@@ -2552,10 +2558,10 @@
         <v>122</v>
       </c>
       <c r="B121" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C121" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
     </row>
     <row r="122" spans="1:3">
@@ -2563,10 +2569,10 @@
         <v>123</v>
       </c>
       <c r="B122" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C122" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
     </row>
     <row r="123" spans="1:3">
@@ -2574,10 +2580,10 @@
         <v>124</v>
       </c>
       <c r="B123" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C123" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
     </row>
     <row r="124" spans="1:3">
@@ -2585,10 +2591,10 @@
         <v>125</v>
       </c>
       <c r="B124" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C124" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
     </row>
     <row r="125" spans="1:3">
@@ -2596,10 +2602,10 @@
         <v>126</v>
       </c>
       <c r="B125" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C125" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
     </row>
     <row r="126" spans="1:3">
@@ -2607,10 +2613,10 @@
         <v>127</v>
       </c>
       <c r="B126" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C126" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="127" spans="1:3">
@@ -2618,10 +2624,10 @@
         <v>128</v>
       </c>
       <c r="B127" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C127" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
     </row>
     <row r="128" spans="1:3">
@@ -2629,10 +2635,10 @@
         <v>129</v>
       </c>
       <c r="B128" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C128" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
     </row>
     <row r="129" spans="1:3">
@@ -2640,10 +2646,10 @@
         <v>130</v>
       </c>
       <c r="B129" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C129" t="s">
-        <v>291</v>
+        <v>279</v>
       </c>
     </row>
     <row r="130" spans="1:3">
@@ -2651,10 +2657,10 @@
         <v>131</v>
       </c>
       <c r="B130" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C130" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
     </row>
     <row r="131" spans="1:3">
@@ -2662,10 +2668,10 @@
         <v>132</v>
       </c>
       <c r="B131" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C131" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
     </row>
     <row r="132" spans="1:3">
@@ -2673,10 +2679,10 @@
         <v>133</v>
       </c>
       <c r="B132" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C132" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="133" spans="1:3">
@@ -2684,10 +2690,10 @@
         <v>134</v>
       </c>
       <c r="B133" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C133" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
     </row>
     <row r="134" spans="1:3">
@@ -2695,10 +2701,10 @@
         <v>135</v>
       </c>
       <c r="B134" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C134" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
     </row>
     <row r="135" spans="1:3">
@@ -2706,10 +2712,10 @@
         <v>136</v>
       </c>
       <c r="B135" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C135" t="s">
-        <v>278</v>
+        <v>288</v>
       </c>
     </row>
     <row r="136" spans="1:3">
@@ -2717,10 +2723,10 @@
         <v>137</v>
       </c>
       <c r="B136" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C136" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="137" spans="1:3">
@@ -2728,10 +2734,10 @@
         <v>138</v>
       </c>
       <c r="B137" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C137" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="138" spans="1:3">
@@ -2739,10 +2745,21 @@
         <v>139</v>
       </c>
       <c r="B138" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C138" t="s">
-        <v>277</v>
+        <v>287</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3">
+      <c r="A139" t="s">
+        <v>140</v>
+      </c>
+      <c r="B139" t="s">
+        <v>278</v>
+      </c>
+      <c r="C139" t="s">
+        <v>279</v>
       </c>
     </row>
   </sheetData>

</xml_diff>